<commit_message>
Updated validation for negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000367/negative/01/data/unit-test-coreid-CG0117-negative.xlsx
+++ b/rules/CORE-000367/negative/01/data/unit-test-coreid-CG0117-negative.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -60,8 +60,21 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -75,6 +88,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -98,13 +129,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,7 +481,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
       <c r="B2" s="4" t="str">
@@ -474,18 +508,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>ta.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Trial Arms</v>
       </c>
     </row>
@@ -498,7 +532,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -520,9 +554,89 @@
         <v>Error value</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>ACME Low Dose</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="2">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>ACME Low Dose</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>ACME High Dose</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="2">
+        <v>15</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>ACTARM</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>[ABSENT]</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -609,221 +723,221 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="5" t="str">
+      <c r="P3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5">
-        <v>50</v>
-      </c>
-      <c r="N4" s="5">
-        <v>50</v>
-      </c>
-      <c r="O4" s="5">
-        <v>50</v>
-      </c>
-      <c r="P4" s="5">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>50</v>
-      </c>
-      <c r="R4" s="5">
-        <v>50</v>
-      </c>
-      <c r="S4" s="5">
-        <v>50</v>
-      </c>
-      <c r="T4" s="5">
-        <v>50</v>
-      </c>
-      <c r="U4" s="5">
-        <v>50</v>
-      </c>
-      <c r="V4" s="5">
-        <v>50</v>
-      </c>
-      <c r="W4" s="5">
-        <v>50</v>
-      </c>
-      <c r="X4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
+        <v>50</v>
+      </c>
+      <c r="K4" s="6">
+        <v>50</v>
+      </c>
+      <c r="L4" s="6">
+        <v>50</v>
+      </c>
+      <c r="M4" s="6">
+        <v>50</v>
+      </c>
+      <c r="N4" s="6">
+        <v>50</v>
+      </c>
+      <c r="O4" s="6">
+        <v>50</v>
+      </c>
+      <c r="P4" s="6">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="6">
+        <v>50</v>
+      </c>
+      <c r="R4" s="6">
+        <v>50</v>
+      </c>
+      <c r="S4" s="6">
+        <v>50</v>
+      </c>
+      <c r="T4" s="6">
+        <v>50</v>
+      </c>
+      <c r="U4" s="6">
+        <v>50</v>
+      </c>
+      <c r="V4" s="6">
+        <v>50</v>
+      </c>
+      <c r="W4" s="6">
+        <v>50</v>
+      </c>
+      <c r="X4" s="6">
         <v>50</v>
       </c>
     </row>
@@ -858,10 +972,10 @@
       <c r="J5" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="K5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L5" s="2" t="str">
+      <c r="K5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4" t="str">
         <v/>
       </c>
       <c r="M5" s="4" t="str">
@@ -894,7 +1008,7 @@
       <c r="V5" s="4" t="str">
         <v>ACME_LOW_D</v>
       </c>
-      <c r="W5" s="4" t="str">
+      <c r="W5" s="7" t="str">
         <v>ACME Low Dose</v>
       </c>
       <c r="X5" s="4" t="str">
@@ -968,7 +1082,7 @@
       <c r="V6" s="4" t="str">
         <v>ACME_LOW_D</v>
       </c>
-      <c r="W6" s="4" t="str">
+      <c r="W6" s="8" t="str">
         <v>ACME Low Dose</v>
       </c>
       <c r="X6" s="4" t="str">
@@ -1006,10 +1120,10 @@
       <c r="J7" s="4" t="str">
         <v>2014-02-13</v>
       </c>
-      <c r="K7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L7" s="2" t="str">
+      <c r="K7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4" t="str">
         <v/>
       </c>
       <c r="M7" s="4" t="str">
@@ -1042,7 +1156,7 @@
       <c r="V7" s="4" t="str">
         <v>ACME_HIGH_D</v>
       </c>
-      <c r="W7" s="4" t="str">
+      <c r="W7" s="8" t="str">
         <v>ACME High Dose</v>
       </c>
       <c r="X7" s="4" t="str">
@@ -1080,10 +1194,10 @@
       <c r="J8" s="4" t="str">
         <v>2014-03-18</v>
       </c>
-      <c r="K8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L8" s="2" t="str">
+      <c r="K8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
       <c r="M8" s="4" t="str">
@@ -1154,10 +1268,10 @@
       <c r="J9" s="4" t="str">
         <v>2013-08-06</v>
       </c>
-      <c r="K9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L9" s="2" t="str">
+      <c r="K9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="4" t="str">
         <v/>
       </c>
       <c r="M9" s="4" t="str">
@@ -1228,10 +1342,10 @@
       <c r="J10" s="4" t="str">
         <v>2013-04-30</v>
       </c>
-      <c r="K10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L10" s="2" t="str">
+      <c r="K10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="4" t="str">
         <v/>
       </c>
       <c r="M10" s="4" t="str">
@@ -1302,10 +1416,10 @@
       <c r="J11" s="4" t="str">
         <v>2013-06-20</v>
       </c>
-      <c r="K11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L11" s="2" t="str">
+      <c r="K11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="4" t="str">
         <v/>
       </c>
       <c r="M11" s="4" t="str">
@@ -1450,10 +1564,10 @@
       <c r="J13" s="4" t="str">
         <v>2013-04-28</v>
       </c>
-      <c r="K13" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L13" s="2" t="str">
+      <c r="K13" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L13" s="4" t="str">
         <v/>
       </c>
       <c r="M13" s="4" t="str">
@@ -1524,10 +1638,10 @@
       <c r="J14" s="4" t="str">
         <v>2013-09-26</v>
       </c>
-      <c r="K14" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L14" s="2" t="str">
+      <c r="K14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L14" s="4" t="str">
         <v/>
       </c>
       <c r="M14" s="4" t="str">
@@ -1598,10 +1712,10 @@
       <c r="J15" s="4" t="str">
         <v>2013-07-05</v>
       </c>
-      <c r="K15" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L15" s="2" t="str">
+      <c r="K15" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L15" s="4" t="str">
         <v/>
       </c>
       <c r="M15" s="4" t="str">
@@ -1672,10 +1786,10 @@
       <c r="J16" s="4" t="str">
         <v>2014-01-28</v>
       </c>
-      <c r="K16" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L16" s="2" t="str">
+      <c r="K16" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L16" s="4" t="str">
         <v/>
       </c>
       <c r="M16" s="4" t="str">
@@ -1820,10 +1934,10 @@
       <c r="J18" s="4" t="str">
         <v>2013-09-18</v>
       </c>
-      <c r="K18" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L18" s="2" t="str">
+      <c r="K18" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L18" s="4" t="str">
         <v/>
       </c>
       <c r="M18" s="4" t="str">
@@ -1876,16 +1990,16 @@
       <c r="D19" s="4" t="str">
         <v>1022</v>
       </c>
-      <c r="E19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H19" s="2" t="str">
+      <c r="E19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H19" s="4" t="str">
         <v/>
       </c>
       <c r="I19" s="4" t="str">
@@ -1894,10 +2008,10 @@
       <c r="J19" s="4" t="str">
         <v>2014-03-17</v>
       </c>
-      <c r="K19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L19" s="2" t="str">
+      <c r="K19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L19" s="4" t="str">
         <v/>
       </c>
       <c r="M19" s="4" t="str">
@@ -1921,16 +2035,16 @@
       <c r="S19" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="U19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="V19" s="2" t="str">
-        <v/>
-      </c>
-      <c r="W19" s="2" t="str">
+      <c r="T19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V19" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W19" s="4" t="str">
         <v/>
       </c>
       <c r="X19" s="4" t="str">
@@ -1968,10 +2082,10 @@
       <c r="J20" s="4" t="str">
         <v>2013-09-22</v>
       </c>
-      <c r="K20" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L20" s="2" t="str">
+      <c r="K20" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L20" s="4" t="str">
         <v/>
       </c>
       <c r="M20" s="4" t="str">
@@ -2042,10 +2156,10 @@
       <c r="J21" s="4" t="str">
         <v>2014-03-08</v>
       </c>
-      <c r="K21" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L21" s="2" t="str">
+      <c r="K21" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L21" s="4" t="str">
         <v/>
       </c>
       <c r="M21" s="4" t="str">
@@ -2116,10 +2230,10 @@
       <c r="J22" s="4" t="str">
         <v>2013-06-03</v>
       </c>
-      <c r="K22" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L22" s="2" t="str">
+      <c r="K22" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L22" s="4" t="str">
         <v/>
       </c>
       <c r="M22" s="4" t="str">
@@ -2203,98 +2317,98 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Planned Order of Element within Arm</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Element Code</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Description of Element</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Branch</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Transition Rule</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Epoch</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
         <v>50</v>
       </c>
     </row>
@@ -2323,7 +2437,7 @@
       <c r="H5" s="4" t="str">
         <v>Randomized to Placebo</v>
       </c>
-      <c r="I5" s="2" t="str">
+      <c r="I5" s="4" t="str">
         <v/>
       </c>
       <c r="J5" s="4" t="str">
@@ -2352,10 +2466,10 @@
       <c r="G6" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="H6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I6" s="2" t="str">
+      <c r="H6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I6" s="4" t="str">
         <v/>
       </c>
       <c r="J6" s="4" t="str">
@@ -2387,7 +2501,7 @@
       <c r="H7" s="4" t="str">
         <v>Randomized to Zanomaline Low Dose</v>
       </c>
-      <c r="I7" s="2" t="str">
+      <c r="I7" s="4" t="str">
         <v/>
       </c>
       <c r="J7" s="4" t="str">
@@ -2416,10 +2530,10 @@
       <c r="G8" s="4" t="str">
         <v>Zanomaline 54 mg</v>
       </c>
-      <c r="H8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I8" s="2" t="str">
+      <c r="H8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I8" s="4" t="str">
         <v/>
       </c>
       <c r="J8" s="4" t="str">
@@ -2451,7 +2565,7 @@
       <c r="H9" s="4" t="str">
         <v>Randomized to Zanomaline High Dose</v>
       </c>
-      <c r="I9" s="2" t="str">
+      <c r="I9" s="4" t="str">
         <v/>
       </c>
       <c r="J9" s="4" t="str">
@@ -2480,10 +2594,10 @@
       <c r="G10" s="4" t="str">
         <v>Zanomaline 54 mg Titration</v>
       </c>
-      <c r="H10" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I10" s="2" t="str">
+      <c r="H10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I10" s="4" t="str">
         <v/>
       </c>
       <c r="J10" s="4" t="str">
@@ -2512,10 +2626,10 @@
       <c r="G11" s="4" t="str">
         <v>Zanomaline 81 mg</v>
       </c>
-      <c r="H11" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I11" s="2" t="str">
+      <c r="H11" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I11" s="4" t="str">
         <v/>
       </c>
       <c r="J11" s="4" t="str">
@@ -2544,10 +2658,10 @@
       <c r="G12" s="4" t="str">
         <v>Zanomaline 54 mg Titration</v>
       </c>
-      <c r="H12" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I12" s="2" t="str">
+      <c r="H12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I12" s="4" t="str">
         <v/>
       </c>
       <c r="J12" s="4" t="str">

</xml_diff>